<commit_message>
Update data validation and backtest reports
</commit_message>
<xml_diff>
--- a/backtest/backtest_report.xlsx
+++ b/backtest/backtest_report.xlsx
@@ -509,35 +509,35 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>100000</v>
       </c>
       <c r="E2" t="n">
-        <v>483676.665958097</v>
+        <v>481041.0341786277</v>
       </c>
       <c r="F2" t="n">
-        <v>3.83676665958097</v>
+        <v>3.810410341786277</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08662553923938554</v>
+        <v>0.08622190271357644</v>
       </c>
       <c r="H2" t="n">
         <v>-0.5881612163209825</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1928442597024633</v>
+        <v>0.1927543824406131</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5259052237133559</v>
+        <v>0.5241381549666437</v>
       </c>
       <c r="K2" t="n">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5606060606060606</v>
+        <v>0.5600403632694249</v>
       </c>
     </row>
     <row r="3">
@@ -553,35 +553,35 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>94311.01051101039</v>
       </c>
       <c r="E3" t="n">
-        <v>1661555.464295391</v>
+        <v>1664489.357320941</v>
       </c>
       <c r="F3" t="n">
-        <v>16.61783120859904</v>
+        <v>16.64893990958372</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1655810982604873</v>
+        <v>0.1655082020847214</v>
       </c>
       <c r="H3" t="n">
         <v>-0.5717061118286524</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2786198211339123</v>
+        <v>0.2784775257578878</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6768608358294521</v>
+        <v>0.6768513901379903</v>
       </c>
       <c r="K3" t="n">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5496417604912999</v>
+        <v>0.5501022494887525</v>
       </c>
     </row>
   </sheetData>
@@ -595,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C991"/>
+  <dimension ref="A1:C992"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13483,6 +13483,19 @@
       </c>
       <c r="C991" t="n">
         <v>-0.02090576188116955</v>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>NIFTY 50</t>
+        </is>
+      </c>
+      <c r="C992" t="n">
+        <v>-0.005449160492885241</v>
       </c>
     </row>
   </sheetData>
@@ -13496,7 +13509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E978"/>
+  <dimension ref="A1:E979"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32089,6 +32102,25 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="979">
+      <c r="A979" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>nifty_pharma</t>
+        </is>
+      </c>
+      <c r="C979" t="n">
+        <v>0.08471276080805046</v>
+      </c>
+      <c r="D979" t="n">
+        <v>0.001765750881384864</v>
+      </c>
+      <c r="E979" s="2" t="n">
+        <v>46276</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>